<commit_message>
fix: revise Control 2.8 Customer Key evidence (cycle 2)
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assessment/templates/exchange-online-admin-checklist.xlsx
+++ b/assessment/templates/exchange-online-admin-checklist.xlsx
@@ -593,12 +593,12 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Does a current manual evidence pack document negotiated TLS handshakes, applicable connector controls, and (where deployed) Customer Key and Key Vault or Managed HSM configuration for Copilot-processed data?</t>
+          <t>Does a current manual evidence pack document negotiated TLS handshakes, applicable connector controls, and (where deployed) the tenant-level multi-workload Customer Key DEP (`MDEP`) from `Get-M365DataAtRestEncryptionPolicy` plus its assignment from `Get-M365DataAtRestEncryptionPolicyAssignment`, onboarding state, and Key Vault or Managed HSM configuration for Copilot-processed data? Treat `Get-DataEncryptionPolicy` as Exchange-mailbox DEP evidence only; it cannot prove Copilot MDEP coverage.</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Timestamped negotiated TLS handshake output for representative Microsoft 365 endpoints, including protocol, cipher suite, and certificate; Exchange connector forced-TLS or mutual-TLS configuration export where the tenant uses those mail-flow paths; Customer Key DEP and Customer Key Onboarding Service validation or enablement state, if Customer Key is deployed; Azure Key Vault Premium or Managed HSM evidence showing two distinct paid subscriptions, one vault or HSM per subscription for each Customer Key scenario, HSM-protected keys, 90-day recovery configuration, and purge protection; Manual Microsoft 365 service-encryption review and applicable Service Trust Portal evidence</t>
+          <t>Timestamped negotiated TLS handshake output for representative Microsoft 365 endpoints, including protocol, cipher suite, and certificate; Exchange connector forced-TLS or mutual-TLS configuration export where the tenant uses those mail-flow paths; Tenant-level multi-workload Customer Key DEP (`MDEP`) policy output from Get-M365DataAtRestEncryptionPolicy and tenant assignment output from Get-M365DataAtRestEncryptionPolicyAssignment, with all returned properties, plus Customer Key Onboarding Service validation or enablement state; Exchange-mailbox DEP output cannot satisfy this Copilot evidence requirement; Azure Key Vault Premium or Managed HSM evidence showing two distinct paid subscriptions, one vault or HSM per subscription for each Customer Key scenario, HSM-protected keys, 90-day recovery configuration, and purge protection; Manual Microsoft 365 service-encryption review and applicable Service Trust Portal evidence</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr"/>

</xml_diff>